<commit_message>
summary table errors handled
</commit_message>
<xml_diff>
--- a/electron/data/portfolio1.xlsx
+++ b/electron/data/portfolio1.xlsx
@@ -435,7 +435,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2025-10-01</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B3" t="str">
         <v>DCR</v>
@@ -444,27 +444,27 @@
         <v>Buy</v>
       </c>
       <c r="D3" t="str">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="E3" t="str">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2025-09-10</v>
+        <v>2025-08-13</v>
       </c>
       <c r="B4" t="str">
-        <v>mebl</v>
+        <v>sazew</v>
       </c>
       <c r="C4" t="str">
         <v>Buy</v>
       </c>
       <c r="D4" t="str">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="E4" t="str">
-        <v>219</v>
+        <v>1400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>